<commit_message>
add images to budget spreadsheet page
</commit_message>
<xml_diff>
--- a/public/growing-forward-monthly-budget.xlsx
+++ b/public/growing-forward-monthly-budget.xlsx
@@ -3,18 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="START HERE" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Dual Paycheck" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Single Paycheck" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="Overview" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="START HERE" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Dual Paycheck" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Single Paycheck" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Overview" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
-  <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="1IqGspxA8TjCRrsyfjEtnV1TX2IdpuNhZ1Qn5Ap0S0Q="/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -297,9 +292,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -529,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -587,6 +583,9 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="15" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -594,6 +593,9 @@
     </xf>
     <xf borderId="5" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -617,10 +619,13 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="4" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="7" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -629,6 +634,12 @@
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="18" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="13" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="5" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -963,7 +974,7 @@
     <xdr:ext cx="5476875" cy="5229225"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="303591829" name="Chart 1"/>
+        <xdr:cNvPr id="1" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -979,6 +990,10 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2565,31 +2580,31 @@
         <v>31</v>
       </c>
       <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="21">
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="22">
         <f t="shared" ref="F5:F12" si="1">IFERROR(IF(B5="",0,B5),0)+IFERROR(IF(D5="",0,D5),0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="22">
         <f t="shared" ref="G5:G12" si="2">F5*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="24">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2599,31 +2614,31 @@
         <v>33</v>
       </c>
       <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="21">
+      <c r="E7" s="21"/>
+      <c r="F7" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="24">
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2633,31 +2648,31 @@
         <v>35</v>
       </c>
       <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="21">
+      <c r="E9" s="21"/>
+      <c r="F9" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24">
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2666,55 +2681,55 @@
       <c r="A11" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="21">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G11" s="21">
+      <c r="G11" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24">
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="26">
+      <c r="B13" s="28">
         <f>SUM(B5:B12)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="26">
+      <c r="C13" s="29"/>
+      <c r="D13" s="28">
         <f>SUM(D5:D12)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="27"/>
-      <c r="F13" s="26">
+      <c r="E13" s="29"/>
+      <c r="F13" s="28">
         <f t="shared" ref="F13:G13" si="3">SUM(F5:F12)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="28">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2734,32 +2749,32 @@
       <c r="A15" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="21">
+      <c r="E15" s="21"/>
+      <c r="F15" s="22">
         <f t="shared" ref="F15:F21" si="4">IFERROR(IF(B15="",0,B15),0)+IFERROR(IF(D15="",0,D15),0)</f>
         <v>0</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="22">
         <f t="shared" ref="G15:G21" si="5">F15*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24">
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2768,32 +2783,32 @@
       <c r="A17" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="21">
+      <c r="E17" s="21"/>
+      <c r="F17" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24">
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2802,32 +2817,32 @@
       <c r="A19" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24">
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2836,38 +2851,38 @@
       <c r="A21" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="21">
+      <c r="E21" s="21"/>
+      <c r="F21" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G21" s="21">
+      <c r="G21" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="28">
         <f>SUM(B15:B21)</f>
         <v>0</v>
       </c>
-      <c r="C22" s="27"/>
-      <c r="D22" s="26">
+      <c r="C22" s="29"/>
+      <c r="D22" s="28">
         <f>SUM(D15:D21)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="27"/>
-      <c r="F22" s="26">
+      <c r="E22" s="29"/>
+      <c r="F22" s="28">
         <f t="shared" ref="F22:G22" si="6">SUM(F15:F21)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="26">
+      <c r="G22" s="28">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2888,31 +2903,31 @@
         <v>50</v>
       </c>
       <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="21">
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="22">
         <f t="shared" ref="F24:F31" si="7">IFERROR(IF(B24="",0,B24),0)+IFERROR(IF(D24="",0,D24),0)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="21">
+      <c r="G24" s="22">
         <f t="shared" ref="G24:G31" si="8">F24*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="24">
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -2921,32 +2936,32 @@
       <c r="A26" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="21">
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G26" s="21">
+      <c r="G26" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="24">
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -2955,32 +2970,32 @@
       <c r="A28" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="21">
+      <c r="E28" s="21"/>
+      <c r="F28" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G28" s="21">
+      <c r="G28" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" ht="16.5" customHeight="1">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="24">
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -2989,55 +3004,55 @@
       <c r="A30" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="21">
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G30" s="21">
+      <c r="G30" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" ht="16.5" customHeight="1">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="24">
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G31" s="24">
+      <c r="G31" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="25" t="s">
+      <c r="A32" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="28">
         <f>SUM(B24:B31)</f>
         <v>0</v>
       </c>
-      <c r="C32" s="27"/>
-      <c r="D32" s="26">
+      <c r="C32" s="29"/>
+      <c r="D32" s="28">
         <f>SUM(D24:D31)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="27"/>
-      <c r="F32" s="26">
+      <c r="E32" s="29"/>
+      <c r="F32" s="28">
         <f t="shared" ref="F32:G32" si="9">SUM(F24:F31)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="26">
+      <c r="G32" s="28">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -3057,32 +3072,32 @@
       <c r="A34" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="21">
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22">
         <f t="shared" ref="F34:F37" si="10">IFERROR(IF(B34="",0,B34),0)+IFERROR(IF(D34="",0,D34),0)</f>
         <v>0</v>
       </c>
-      <c r="G34" s="21">
+      <c r="G34" s="22">
         <f t="shared" ref="G34:G37" si="11">F34*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="23"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="24">
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="26">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="26">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -3091,49 +3106,49 @@
       <c r="A36" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="21">
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="22">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="G36" s="21">
+      <c r="G36" s="22">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="24">
+      <c r="B37" s="25"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="26">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="G37" s="24">
+      <c r="G37" s="26">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="26">
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="28">
         <f t="shared" ref="F38:G38" si="12">SUM(F34:F37)</f>
         <v>0</v>
       </c>
-      <c r="G38" s="26">
+      <c r="G38" s="28">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
@@ -3150,7 +3165,7 @@
       <c r="G39" s="4"/>
     </row>
     <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="28" t="s">
+      <c r="A40" s="30" t="s">
         <v>66</v>
       </c>
       <c r="B40" s="3"/>
@@ -3161,55 +3176,55 @@
       <c r="G40" s="4"/>
     </row>
     <row r="41" ht="16.5" customHeight="1">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="B41" s="30"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31">
-        <f>IF(F41="",0,F41*26)</f>
+      <c r="B41" s="32"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="34">
+        <f>F41*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="B42" s="27"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="26">
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="28">
         <f>B13+B22+B32</f>
         <v>0</v>
       </c>
-      <c r="G42" s="26">
-        <f>(B13+B22+B32)*26</f>
+      <c r="G42" s="28">
+        <f>(B13+B22+B32)*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="21.75" customHeight="1">
-      <c r="A43" s="32" t="s">
+      <c r="A43" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="B43" s="33"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="35">
+      <c r="B43" s="36"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="37"/>
+      <c r="F43" s="38">
         <f t="shared" ref="F43:G43" si="13">F41-F42</f>
         <v>0</v>
       </c>
-      <c r="G43" s="35">
+      <c r="G43" s="38">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="44" ht="21.75" customHeight="1">
-      <c r="A44" s="28" t="s">
+      <c r="A44" s="30" t="s">
         <v>70</v>
       </c>
       <c r="B44" s="3"/>
@@ -3220,55 +3235,55 @@
       <c r="G44" s="4"/>
     </row>
     <row r="45" ht="16.5" customHeight="1">
-      <c r="A45" s="29" t="s">
+      <c r="A45" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31">
-        <f>IF(F45="",0,F45*26)</f>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34">
+        <f>F45*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" ht="16.5" customHeight="1">
-      <c r="A46" s="25" t="s">
+      <c r="A46" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="B46" s="27"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="26">
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="28">
         <f>D13+D22+D32</f>
         <v>0</v>
       </c>
-      <c r="G46" s="26">
-        <f>(D13+D22+D32)*26</f>
+      <c r="G46" s="28">
+        <f>(D13+D22+D32)*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" ht="21.75" customHeight="1">
-      <c r="A47" s="32" t="s">
+      <c r="A47" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="33"/>
-      <c r="C47" s="33"/>
-      <c r="D47" s="33"/>
-      <c r="E47" s="34"/>
-      <c r="F47" s="35">
+      <c r="B47" s="36"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="38">
         <f t="shared" ref="F47:G47" si="14">F45-F46</f>
         <v>0</v>
       </c>
-      <c r="G47" s="35">
+      <c r="G47" s="38">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
     </row>
     <row r="48" ht="21.75" customHeight="1">
-      <c r="A48" s="28" t="s">
+      <c r="A48" s="30" t="s">
         <v>74</v>
       </c>
       <c r="B48" s="3"/>
@@ -3279,52 +3294,52 @@
       <c r="G48" s="4"/>
     </row>
     <row r="49" ht="16.5" customHeight="1">
-      <c r="A49" s="29" t="s">
+      <c r="A49" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="30"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="31">
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="39">
         <f t="shared" ref="F49:G49" si="15">F41+F45</f>
         <v>0</v>
       </c>
-      <c r="G49" s="31">
+      <c r="G49" s="39">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="16.5" customHeight="1">
-      <c r="A50" s="25" t="s">
+      <c r="A50" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-      <c r="F50" s="26">
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="29"/>
+      <c r="F50" s="28">
         <f t="shared" ref="F50:G50" si="16">F13+F22+F32+F38</f>
         <v>0</v>
       </c>
-      <c r="G50" s="26">
+      <c r="G50" s="28">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
     </row>
     <row r="51" ht="21.75" customHeight="1">
-      <c r="A51" s="32" t="s">
+      <c r="A51" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="B51" s="33"/>
-      <c r="C51" s="33"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="35">
+      <c r="B51" s="36"/>
+      <c r="C51" s="36"/>
+      <c r="D51" s="36"/>
+      <c r="E51" s="37"/>
+      <c r="F51" s="38">
         <f t="shared" ref="F51:G51" si="17">F49-F50</f>
         <v>0</v>
       </c>
-      <c r="G51" s="35">
+      <c r="G51" s="38">
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
@@ -4395,27 +4410,27 @@
         <v>31</v>
       </c>
       <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21">
+      <c r="C5" s="21"/>
+      <c r="D5" s="22">
         <f t="shared" ref="D5:D12" si="1">IFERROR(IF(B5="",0,B5),0)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="22">
         <f t="shared" ref="E5:E12" si="2">D5*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="24">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -4425,27 +4440,27 @@
         <v>33</v>
       </c>
       <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="21">
+      <c r="C7" s="21"/>
+      <c r="D7" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="24">
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -4455,27 +4470,27 @@
         <v>35</v>
       </c>
       <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="21">
+      <c r="C9" s="21"/>
+      <c r="D9" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24">
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -4484,46 +4499,46 @@
       <c r="A11" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="21">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="24">
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="26">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="26">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="26">
+      <c r="B13" s="28">
         <f>SUM(B5:B12)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="26">
+      <c r="C13" s="29"/>
+      <c r="D13" s="28">
         <f t="shared" ref="D13:E13" si="3">SUM(D5:D12)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="28">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -4542,27 +4557,27 @@
         <v>41</v>
       </c>
       <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21">
+      <c r="C15" s="21"/>
+      <c r="D15" s="22">
         <f t="shared" ref="D15:D21" si="4">IFERROR(IF(B15="",0,B15),0)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="22">
         <f t="shared" ref="E15:E21" si="5">D15*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24">
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4571,28 +4586,28 @@
       <c r="A17" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="21">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24">
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4602,27 +4617,27 @@
         <v>45</v>
       </c>
       <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21">
+      <c r="C19" s="21"/>
+      <c r="D19" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24">
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="26">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="26">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4631,31 +4646,31 @@
       <c r="A21" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21">
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="E21" s="21">
+      <c r="E21" s="22">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="28">
         <f>SUM(B15:B21)</f>
         <v>0</v>
       </c>
-      <c r="C22" s="27"/>
-      <c r="D22" s="26">
+      <c r="C22" s="29"/>
+      <c r="D22" s="28">
         <f t="shared" ref="D22:E22" si="6">SUM(D15:D21)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="28">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -4674,27 +4689,27 @@
         <v>50</v>
       </c>
       <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21">
+      <c r="C24" s="21"/>
+      <c r="D24" s="22">
         <f t="shared" ref="D24:D31" si="7">IFERROR(IF(B24="",0,B24),0)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="21">
+      <c r="E24" s="22">
         <f t="shared" ref="E24:E31" si="8">D24*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24">
+      <c r="B25" s="24"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -4703,28 +4718,28 @@
       <c r="A26" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21">
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E26" s="21">
+      <c r="E26" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="24">
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E27" s="24">
+      <c r="E27" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -4733,28 +4748,28 @@
       <c r="A28" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="21">
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E28" s="21">
+      <c r="E28" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" ht="16.5" customHeight="1">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="24">
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E29" s="24">
+      <c r="E29" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -4763,46 +4778,46 @@
       <c r="A30" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="21">
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="22">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="22">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" ht="16.5" customHeight="1">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="24">
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="26">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="E31" s="24">
+      <c r="E31" s="26">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="25" t="s">
+      <c r="A32" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="26">
+      <c r="B32" s="28">
         <f>SUM(B24:B31)</f>
         <v>0</v>
       </c>
-      <c r="C32" s="27"/>
-      <c r="D32" s="26">
+      <c r="C32" s="29"/>
+      <c r="D32" s="28">
         <f t="shared" ref="D32:E32" si="9">SUM(D24:D31)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="26">
+      <c r="E32" s="28">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -4820,28 +4835,28 @@
       <c r="A34" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="21">
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="22">
         <f t="shared" ref="D34:D37" si="10">IFERROR(IF(B34="",0,B34),0)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="21">
+      <c r="E34" s="22">
         <f t="shared" ref="E34:E37" si="11">D34*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="23"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="24">
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="26">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="E35" s="24">
+      <c r="E35" s="26">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -4850,43 +4865,43 @@
       <c r="A36" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="21">
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="22">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="E36" s="21">
+      <c r="E36" s="22">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="24">
+      <c r="B37" s="25"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="26">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="26">
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="28">
         <f t="shared" ref="D38:E38" si="12">SUM(D34:D37)</f>
         <v>0</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="28">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
@@ -4901,43 +4916,43 @@
       <c r="E39" s="4"/>
     </row>
     <row r="40" ht="16.5" customHeight="1">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="B40" s="30"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31">
+      <c r="B40" s="32"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="34">
         <f>D40*12</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="26">
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="28">
         <f t="shared" ref="D41:E41" si="13">D13+D22+D32+D38</f>
         <v>0</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="28">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="42" ht="21.75" customHeight="1">
-      <c r="A42" s="32" t="s">
+      <c r="A42" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="33"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="35">
+      <c r="B42" s="36"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="38">
         <f t="shared" ref="D42:E42" si="14">D40-D41</f>
         <v>0</v>
       </c>
-      <c r="E42" s="35">
+      <c r="E42" s="38">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
@@ -5962,46 +5977,46 @@
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="1">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B4" s="42">
         <f>'Dual Paycheck'!F13</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="39">
+      <c r="B5" s="44">
         <f>'Dual Paycheck'!F22</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="18.0" customHeight="1">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="42">
         <f>'Dual Paycheck'!F32</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="18.0" customHeight="1">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="44">
         <f>'Dual Paycheck'!F38</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="18.0" customHeight="1">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="42">
         <f>'Dual Paycheck'!F51</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
restructure learn section to /learn route
</commit_message>
<xml_diff>
--- a/public/growing-forward-monthly-budget.xlsx
+++ b/public/growing-forward-monthly-budget.xlsx
@@ -3183,7 +3183,9 @@
       <c r="C41" s="33"/>
       <c r="D41" s="33"/>
       <c r="E41" s="33"/>
-      <c r="F41" s="34"/>
+      <c r="F41" s="34">
+        <v>0.0</v>
+      </c>
       <c r="G41" s="34">
         <f>F41*12</f>
         <v>0</v>
@@ -3242,7 +3244,9 @@
       <c r="C45" s="33"/>
       <c r="D45" s="33"/>
       <c r="E45" s="33"/>
-      <c r="F45" s="34"/>
+      <c r="F45" s="34">
+        <v>0.0</v>
+      </c>
       <c r="G45" s="34">
         <f>F45*12</f>
         <v>0</v>
@@ -4921,7 +4925,9 @@
       </c>
       <c r="B40" s="32"/>
       <c r="C40" s="33"/>
-      <c r="D40" s="40"/>
+      <c r="D40" s="40">
+        <v>0.0</v>
+      </c>
       <c r="E40" s="34">
         <f>D40*12</f>
         <v>0</v>

</xml_diff>